<commit_message>
Fix Edit Month/Payment modal to accurately load recorded payment amount and enforce single payment entry per lease contract per month
</commit_message>
<xml_diff>
--- a/Property_Rent_Data_Model.xlsx
+++ b/Property_Rent_Data_Model.xlsx
@@ -8717,16 +8717,16 @@
         <v>3399918.74</v>
       </c>
       <c r="D86">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="E86">
         <v>0</v>
       </c>
       <c r="F86">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="G86">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="H86" t="str">
         <v>Yes</v>
@@ -8749,7 +8749,7 @@
         <v>2026-06</v>
       </c>
       <c r="C87">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="D87">
         <v>0</v>
@@ -8761,7 +8761,7 @@
         <v>0</v>
       </c>
       <c r="G87">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="H87" t="str">
         <v>Yes</v>
@@ -8784,7 +8784,7 @@
         <v>2026-07</v>
       </c>
       <c r="C88">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="D88">
         <v>0</v>
@@ -8796,7 +8796,7 @@
         <v>0</v>
       </c>
       <c r="G88">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="H88" t="str">
         <v>Yes</v>
@@ -8819,7 +8819,7 @@
         <v>2026-08</v>
       </c>
       <c r="C89">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="D89">
         <v>0</v>
@@ -8831,7 +8831,7 @@
         <v>0</v>
       </c>
       <c r="G89">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="H89" t="str">
         <v>Yes</v>
@@ -8854,7 +8854,7 @@
         <v>2026-09</v>
       </c>
       <c r="C90">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="D90">
         <v>0</v>
@@ -8866,7 +8866,7 @@
         <v>0</v>
       </c>
       <c r="G90">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="H90" t="str">
         <v>Yes</v>
@@ -8889,7 +8889,7 @@
         <v>2026-10</v>
       </c>
       <c r="C91">
-        <v>3399918.74</v>
+        <v>3419918.74</v>
       </c>
       <c r="D91">
         <v>3262426</v>
@@ -8901,7 +8901,7 @@
         <v>3262426</v>
       </c>
       <c r="G91">
-        <v>6662344.74</v>
+        <v>6682344.74</v>
       </c>
       <c r="H91" t="str">
         <v>Yes</v>

</xml_diff>

<commit_message>
Fix saving rent amount for any month paid for different from accounting month
</commit_message>
<xml_diff>
--- a/Property_Rent_Data_Model.xlsx
+++ b/Property_Rent_Data_Model.xlsx
@@ -837,7 +837,7 @@
         <v>PaymentReceipts</v>
       </c>
       <c r="B39">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="40">
@@ -845,7 +845,7 @@
         <v>PaymentAllocations</v>
       </c>
       <c r="B40">
-        <v>703</v>
+        <v>708</v>
       </c>
     </row>
     <row r="41">
@@ -893,7 +893,7 @@
         <v>TOTAL</v>
       </c>
       <c r="B46">
-        <v>2908</v>
+        <v>2915</v>
       </c>
     </row>
   </sheetData>
@@ -8472,16 +8472,16 @@
         <v>2545021.74</v>
       </c>
       <c r="D79">
-        <v>348016</v>
+        <v>316016</v>
       </c>
       <c r="E79">
         <v>71548</v>
       </c>
       <c r="F79">
-        <v>276468</v>
+        <v>244468</v>
       </c>
       <c r="G79">
-        <v>2821489.74</v>
+        <v>2789489.74</v>
       </c>
       <c r="H79" t="str">
         <v>Yes</v>
@@ -8504,7 +8504,7 @@
         <v>2025-11</v>
       </c>
       <c r="C80">
-        <v>2821489.74</v>
+        <v>2789489.74</v>
       </c>
       <c r="D80">
         <v>185000</v>
@@ -8516,7 +8516,7 @@
         <v>118500</v>
       </c>
       <c r="G80">
-        <v>2939989.74</v>
+        <v>2907989.74</v>
       </c>
       <c r="H80" t="str">
         <v>Yes</v>
@@ -8539,7 +8539,7 @@
         <v>2025-12</v>
       </c>
       <c r="C81">
-        <v>2939989.74</v>
+        <v>2907989.74</v>
       </c>
       <c r="D81">
         <v>715000</v>
@@ -8551,7 +8551,7 @@
         <v>670199</v>
       </c>
       <c r="G81">
-        <v>3610188.74</v>
+        <v>3578188.74</v>
       </c>
       <c r="H81" t="str">
         <v>Yes</v>
@@ -8577,16 +8577,16 @@
         <v>5643188.74</v>
       </c>
       <c r="D82">
-        <v>581050</v>
+        <v>549050</v>
       </c>
       <c r="E82">
         <v>13670</v>
       </c>
       <c r="F82">
-        <v>567380</v>
+        <v>535380</v>
       </c>
       <c r="G82">
-        <v>6210568.74</v>
+        <v>6178568.74</v>
       </c>
       <c r="H82" t="str">
         <v>Yes</v>
@@ -8609,7 +8609,7 @@
         <v>2026-02</v>
       </c>
       <c r="C83">
-        <v>6210568.74</v>
+        <v>6178568.74</v>
       </c>
       <c r="D83">
         <v>0</v>
@@ -8621,7 +8621,7 @@
         <v>-4800</v>
       </c>
       <c r="G83">
-        <v>6205768.74</v>
+        <v>6173768.74</v>
       </c>
       <c r="H83" t="str">
         <v>Yes</v>
@@ -8644,19 +8644,19 @@
         <v>2026-03</v>
       </c>
       <c r="C84">
-        <v>6205768.74</v>
+        <v>6173768.74</v>
       </c>
       <c r="D84">
-        <v>240000</v>
+        <v>258000</v>
       </c>
       <c r="E84">
         <v>2874350</v>
       </c>
       <c r="F84">
-        <v>-2634350</v>
+        <v>-2616350</v>
       </c>
       <c r="G84">
-        <v>3571418.74</v>
+        <v>3557418.74</v>
       </c>
       <c r="H84" t="str">
         <v>Yes</v>
@@ -8679,7 +8679,7 @@
         <v>2026-04</v>
       </c>
       <c r="C85">
-        <v>3571418.74</v>
+        <v>3557418.74</v>
       </c>
       <c r="D85">
         <v>28500</v>
@@ -8691,7 +8691,7 @@
         <v>-171500</v>
       </c>
       <c r="G85">
-        <v>3399918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="H85" t="str">
         <v>Yes</v>
@@ -8714,19 +8714,19 @@
         <v>2026-05</v>
       </c>
       <c r="C86">
-        <v>3399918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="D86">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="E86">
         <v>0</v>
       </c>
       <c r="F86">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="G86">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="H86" t="str">
         <v>Yes</v>
@@ -8749,7 +8749,7 @@
         <v>2026-06</v>
       </c>
       <c r="C87">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="D87">
         <v>0</v>
@@ -8761,7 +8761,7 @@
         <v>0</v>
       </c>
       <c r="G87">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="H87" t="str">
         <v>Yes</v>
@@ -8784,7 +8784,7 @@
         <v>2026-07</v>
       </c>
       <c r="C88">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="D88">
         <v>0</v>
@@ -8796,7 +8796,7 @@
         <v>0</v>
       </c>
       <c r="G88">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="H88" t="str">
         <v>Yes</v>
@@ -8819,7 +8819,7 @@
         <v>2026-08</v>
       </c>
       <c r="C89">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="D89">
         <v>0</v>
@@ -8831,7 +8831,7 @@
         <v>0</v>
       </c>
       <c r="G89">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="H89" t="str">
         <v>Yes</v>
@@ -8854,7 +8854,7 @@
         <v>2026-09</v>
       </c>
       <c r="C90">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="D90">
         <v>0</v>
@@ -8866,7 +8866,7 @@
         <v>0</v>
       </c>
       <c r="G90">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="H90" t="str">
         <v>Yes</v>
@@ -8889,19 +8889,19 @@
         <v>2026-10</v>
       </c>
       <c r="C91">
-        <v>3419918.74</v>
+        <v>3385918.74</v>
       </c>
       <c r="D91">
-        <v>3262426</v>
+        <v>3412426</v>
       </c>
       <c r="E91">
         <v>0</v>
       </c>
       <c r="F91">
-        <v>3262426</v>
+        <v>3412426</v>
       </c>
       <c r="G91">
-        <v>6682344.74</v>
+        <v>6798344.74</v>
       </c>
       <c r="H91" t="str">
         <v>Yes</v>
@@ -52094,7 +52094,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>[Showing 100 of 701 total records]</v>
+        <v>[Showing 100 of 703 total records]</v>
       </c>
     </row>
     <row r="3">
@@ -56566,7 +56566,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>[Showing 100 of 703 total records]</v>
+        <v>[Showing 100 of 708 total records]</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Show accurate Month Paid For matching Edit modal and implement row and cell arrow key navigation
</commit_message>
<xml_diff>
--- a/Property_Rent_Data_Model.xlsx
+++ b/Property_Rent_Data_Model.xlsx
@@ -845,7 +845,7 @@
         <v>PaymentAllocations</v>
       </c>
       <c r="B40">
-        <v>708</v>
+        <v>711</v>
       </c>
     </row>
     <row r="41">
@@ -893,7 +893,7 @@
         <v>TOTAL</v>
       </c>
       <c r="B46">
-        <v>2915</v>
+        <v>2918</v>
       </c>
     </row>
   </sheetData>
@@ -8892,16 +8892,16 @@
         <v>3385918.74</v>
       </c>
       <c r="D91">
-        <v>3412426</v>
+        <v>3487426</v>
       </c>
       <c r="E91">
         <v>0</v>
       </c>
       <c r="F91">
-        <v>3412426</v>
+        <v>3487426</v>
       </c>
       <c r="G91">
-        <v>6798344.74</v>
+        <v>6873344.74</v>
       </c>
       <c r="H91" t="str">
         <v>Yes</v>
@@ -56566,7 +56566,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>[Showing 100 of 708 total records]</v>
+        <v>[Showing 100 of 711 total records]</v>
       </c>
     </row>
     <row r="3">

</xml_diff>